<commit_message>
truck availability in node_metrics_paper.xlsx
</commit_message>
<xml_diff>
--- a/southern_europe/italy_data/network_capex_metrics/pipeline_size_class_connections.xlsx
+++ b/southern_europe/italy_data/network_capex_metrics/pipeline_size_class_connections.xlsx
@@ -3427,7 +3427,7 @@
         <v>1</v>
       </c>
       <c r="AA21" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB21" t="n">
         <v>1</v>
@@ -3570,7 +3570,7 @@
         <v>1</v>
       </c>
       <c r="Z22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA22" t="n">
         <v>1</v>
@@ -5507,7 +5507,7 @@
         <v>1</v>
       </c>
       <c r="AM35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AN35" t="n">
         <v>1</v>

</xml_diff>